<commit_message>
feat(dictionary): add prompt with audited workflow
</commit_message>
<xml_diff>
--- a/exports/dictionary_index.xlsx
+++ b/exports/dictionary_index.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J20"/>
+  <dimension ref="A1:J40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -434,7 +434,7 @@
     <col width="16" customWidth="1" min="6" max="6"/>
     <col width="10" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="59" customWidth="1" min="9" max="9"/>
+    <col width="60" customWidth="1" min="9" max="9"/>
     <col width="13" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
@@ -570,7 +570,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>entry_spec_v1</t>
+          <t>entry_spec_v5</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -580,10 +580,14 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr"/>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>revised after independent v5 review; corrected marine-insurance notice and total-loss wording; qualified rare abandoned adjective usage; corrected legal-jurisdiction and decay-register wording; corrected career/habit policy and abandoned-plan examples</t>
+        </is>
+      </c>
       <c r="J3" t="inlineStr">
         <is>
           <t>true</t>
@@ -666,7 +670,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>entry_spec_v1</t>
+          <t>entry_spec_v5</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -676,10 +680,14 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr"/>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>rechecked under current entry_spec_v5 and one context-free cold review; clarified base sufficiency versus contextual lukewarm evaluation; qualified pronunciation and -ate variation; expanded adequately/inadequacy and enough nuance; qualified legal consideration and remedy phrases; all candidates adjudicated with no holds; full reinspection passed</t>
+        </is>
+      </c>
       <c r="J5" t="inlineStr">
         <is>
           <t>true</t>
@@ -762,7 +770,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>entry_spec_v1</t>
+          <t>entry_spec_v5</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -772,10 +780,14 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr"/>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>rechecked after context-free zero-based evaluation; corrected additive A/B explanation and translations</t>
+        </is>
+      </c>
       <c r="J7" t="inlineStr">
         <is>
           <t>true</t>
@@ -858,7 +870,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>entry_spec_v1</t>
+          <t>entry_spec_v5</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -868,10 +880,14 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr"/>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>cycle-006 strict three-party audit PASS; corrected supply-network overgeneralization mathematical action direction generalized-function relation medical coverage and electricity transmission boundary; retained PyPA's documented distribution-package terminology variation; cycle-005 remains preserved and superseded</t>
+        </is>
+      </c>
       <c r="J9" t="inlineStr">
         <is>
           <t>true</t>
@@ -1146,7 +1162,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>entry_spec_v1</t>
+          <t>entry_spec_v5</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1156,10 +1172,14 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
-        </is>
-      </c>
-      <c r="I15" t="inlineStr"/>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>zero-based v5 recheck; corrected caster/forecast wording; corrected casting frames; clarified computer coercion and type-conversion terminology; separated cast-of senses; qualified contrast expressions; refreshed article hash and audit</t>
+        </is>
+      </c>
       <c r="J15" t="inlineStr">
         <is>
           <t>true</t>
@@ -1242,7 +1262,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>entry_spec_v1</t>
+          <t>entry_spec_v5</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1252,10 +1272,14 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
-        </is>
-      </c>
-      <c r="I17" t="inlineStr"/>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>v5 normal and context-free cold review passed; corrected patent-law synonym coverage; blind inventory sealed before reconciliation; final target relation evidence semantic and source-first gates passed</t>
+        </is>
+      </c>
       <c r="J17" t="inlineStr">
         <is>
           <t>true</t>
@@ -1290,7 +1314,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>entry_spec_v1</t>
+          <t>entry_spec_v5</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1300,10 +1324,14 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
-        </is>
-      </c>
-      <c r="I18" t="inlineStr"/>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>corrected general extent-severity-impact evaluation</t>
+        </is>
+      </c>
       <c r="J18" t="inlineStr">
         <is>
           <t>true</t>
@@ -1409,6 +1437,1046 @@
         </is>
       </c>
       <c r="J20" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>approximately</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>word</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>checked</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="E21" s="1" t="inlineStr">
+        <is>
+          <t>entries/a/approximately.md</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>entry_spec_v5</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>revised after zero-base usage review; restored explicit approximate adjective/verb pronunciation and syllabification; broadened adjective/participle approximation patterns; clarified close to</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>embrace</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>word</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>checked</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="E22" s="1" t="inlineStr">
+        <is>
+          <t>entries/e/embrace.md</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>entry_spec_v5</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>repository-wide v5 notation scan; canonicalized placeholders and current heading</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>revere</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>word</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>checked</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+      <c r="E23" s="1" t="inlineStr">
+        <is>
+          <t>entries/r/revere.md</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>entry_spec_v5</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>repository-wide v5 notation scan; canonicalized placeholders and current heading</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>endorsement</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>word</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>checked</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="E24" s="1" t="inlineStr">
+        <is>
+          <t>entries/e/endorsement.md</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>entry_spec_v5</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>revised all six review findings; canonicalized notation and strengthened validator coverage</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>overwhelm</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>word</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>checked</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="E25" s="1" t="inlineStr">
+        <is>
+          <t>entries/o/overwhelm.md</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>entry_spec_v5</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>revised after final grammar-pattern slot review and independently zero-base checked under v5</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>device</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>word</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>checked</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="E26" s="1" t="inlineStr">
+        <is>
+          <t>entries/d/device.md</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>entry_spec_v5</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>v5 normal review and context-free cold review passed; blind final inventory sealed before reconciliation; all targets</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>subsequent</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>word</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>checked</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="E27" s="1" t="inlineStr">
+        <is>
+          <t>entries/s/subsequent.md</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>entry_spec_v5</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>v5 normal and cold reviews passed; blind inventory sealed before reconciliation; final target</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>devise</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>word</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>checked</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
+      <c r="E28" s="1" t="inlineStr">
+        <is>
+          <t>entries/d/devise.md</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>entry_spec_v5</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>cycle-003 PASS: consolidated legal noun senses and qualified traditional/current general devise</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>incorporate</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>word</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>checked</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="E29" s="1" t="inlineStr">
+        <is>
+          <t>entries/i/incorporate.md</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>entry_spec_v5</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>v5 normal and context-free cold review passed; blind final inventory sealed before reconciliation; integration</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>privilege</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>word</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>checked</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
+      <c r="E30" s="1" t="inlineStr">
+        <is>
+          <t>entries/p/privilege.md</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>entry_spec_v5</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>v5 normal and context-free cold review passed; blind final inventory sealed before reconciliation; source-first inventory</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>eliminate</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>word</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>checked</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="E31" s="1" t="inlineStr">
+        <is>
+          <t>entries/e/eliminate.md</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>entry_spec_v5</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>follow-up cycle passed; corrected limen/limit etymology</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>retain</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>word</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>checked</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>31</t>
+        </is>
+      </c>
+      <c r="E32" s="1" t="inlineStr">
+        <is>
+          <t>entries/r/retain.md</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>entry_spec_v5</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>v5 revision; cycle-004 chronology-compliant reviews and blind reconciliation passed</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>perceive</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>word</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>checked</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>32</t>
+        </is>
+      </c>
+      <c r="E33" s="1" t="inlineStr">
+        <is>
+          <t>entries/p/perceive.md</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>entry_spec_v5</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>v5 cycle-003 final reconciliation passed; blind seal preceded reconciliation; source-first inventory</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>criterion</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>word</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>checked</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>33</t>
+        </is>
+      </c>
+      <c r="E34" s="1" t="inlineStr">
+        <is>
+          <t>entries/c/criterion.md</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>entry_spec_v5</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>v5 normal/cold/post-cold/blind/final audit passed; 47 targets</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>deserve</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>word</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>checked</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>34</t>
+        </is>
+      </c>
+      <c r="E35" s="1" t="inlineStr">
+        <is>
+          <t>entries/d/deserve.md</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>entry_spec_v5</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>v5 source-first inventory and independent reviews passed; blind seal completed before final reconciliation</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>assert</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>word</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>checked</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
+      </c>
+      <c r="E36" s="1" t="inlineStr">
+        <is>
+          <t>entries/a/assert.md</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>entry_spec_v5</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>source-first inventory complete; normal</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>consistent</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>word</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>checked</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>36</t>
+        </is>
+      </c>
+      <c r="E37" s="1" t="inlineStr">
+        <is>
+          <t>entries/c/consistent.md</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>entry_spec_v5</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>source-first inventory complete; normal</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>extensive</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>word</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>checked</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>37</t>
+        </is>
+      </c>
+      <c r="E38" s="1" t="inlineStr">
+        <is>
+          <t>entries/e/extensive.md</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>entry_spec_v5</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>source-first v2</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>distinct</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>word</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>checked</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>38</t>
+        </is>
+      </c>
+      <c r="E39" s="1" t="inlineStr">
+        <is>
+          <t>entries/d/distinct.md</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>entry_spec_v5</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>process-refactor-v1 E2E passed v6 checker context-free cold review sealed final blind and generated final audit</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>prompt</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>word</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>checked</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>39</t>
+        </is>
+      </c>
+      <c r="E40" s="1" t="inlineStr">
+        <is>
+          <t>entries/p/prompt.md</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>entry_spec_v5</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>extended source-first inventory; normal/cold/final-blind reviews</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
         <is>
           <t>true</t>
         </is>
@@ -1435,6 +2503,26 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E18" r:id="rId17"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E19" r:id="rId18"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E20" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E21" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E22" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E23" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E24" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E25" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E26" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E27" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E28" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E29" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E30" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E31" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E32" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E33" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E34" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E35" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E36" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E37" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E38" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E39" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E40" r:id="rId39"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: finalize conservation audit status and exports
</commit_message>
<xml_diff>
--- a/exports/dictionary_index.xlsx
+++ b/exports/dictionary_index.xlsx
@@ -423,12 +423,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J40"/>
+  <dimension ref="A1:J45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
     <col width="29" customWidth="1" min="5" max="5"/>
     <col width="16" customWidth="1" min="6" max="6"/>
@@ -2477,6 +2477,266 @@
         </is>
       </c>
       <c r="J40" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>pursue</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>word</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>checked</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="E41" s="1" t="inlineStr">
+        <is>
+          <t>entries/p/pursue.md</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>entry_spec_v5</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>external review revision; corrected sense 5 romantic examples; aligned hotly pursue with physical chase; improved sense 6 example and translations; revised audit passed</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>yield</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>word</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>needs_review</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>41</t>
+        </is>
+      </c>
+      <c r="E42" s="1" t="inlineStr">
+        <is>
+          <t>entries/y/yield.md</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>entry_spec_v5</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>previous review invalidated by B1-B4 liveness checks; mode-I acceptance pending</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>assume</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>word</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>checked</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>42</t>
+        </is>
+      </c>
+      <c r="E43" s="1" t="inlineStr">
+        <is>
+          <t>entries/a/assume.md</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>entry_spec_v5</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>source-first inventory; seven checker passes; context-free cold review; blind seal; final reconciliation; 130 targets and 95 relations; 28 source facts</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>genuine</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>word</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>checked</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>43</t>
+        </is>
+      </c>
+      <c r="E44" s="1" t="inlineStr">
+        <is>
+          <t>entries/g/genuine.md</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>entry_spec_v5</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>source-first v2 inventory; seven checker passes; context-free cold review; blind seal; final reconciliation; 89 targets and 51 relations; 24 source facts</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>conservation</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>word</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>checked</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>44</t>
+        </is>
+      </c>
+      <c r="E45" s="1" t="inlineStr">
+        <is>
+          <t>entries/c/conservation.md</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>entry_spec_v5</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>source-first v2 inventory; seven checker passes; context-free cold review; blind seal; final reconciliation; 86 targets and 53 relations; 24 source facts</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
         <is>
           <t>true</t>
         </is>
@@ -2523,6 +2783,11 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E38" r:id="rId37"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E39" r:id="rId38"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E40" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E41" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E42" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E43" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E44" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E45" r:id="rId44"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: add conservation dictionary entry (#119)
Add the v5 conservation entry with audited definitions, queue metadata, and exports.
</commit_message>
<xml_diff>
--- a/exports/dictionary_index.xlsx
+++ b/exports/dictionary_index.xlsx
@@ -423,12 +423,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J40"/>
+  <dimension ref="A1:J45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
     <col width="29" customWidth="1" min="5" max="5"/>
     <col width="16" customWidth="1" min="6" max="6"/>
@@ -2477,6 +2477,266 @@
         </is>
       </c>
       <c r="J40" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>pursue</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>word</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>checked</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="E41" s="1" t="inlineStr">
+        <is>
+          <t>entries/p/pursue.md</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>entry_spec_v5</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>external review revision; corrected sense 5 romantic examples; aligned hotly pursue with physical chase; improved sense 6 example and translations; revised audit passed</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>yield</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>word</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>needs_review</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>41</t>
+        </is>
+      </c>
+      <c r="E42" s="1" t="inlineStr">
+        <is>
+          <t>entries/y/yield.md</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>entry_spec_v5</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>previous review invalidated by B1-B4 liveness checks; mode-I acceptance pending</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>assume</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>word</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>checked</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>42</t>
+        </is>
+      </c>
+      <c r="E43" s="1" t="inlineStr">
+        <is>
+          <t>entries/a/assume.md</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>entry_spec_v5</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>source-first inventory; seven checker passes; context-free cold review; blind seal; final reconciliation; 130 targets and 95 relations; 28 source facts</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>genuine</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>word</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>checked</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>43</t>
+        </is>
+      </c>
+      <c r="E44" s="1" t="inlineStr">
+        <is>
+          <t>entries/g/genuine.md</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>entry_spec_v5</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>source-first v2 inventory; seven checker passes; context-free cold review; blind seal; final reconciliation; 89 targets and 51 relations; 24 source facts</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>conservation</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>word</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>checked</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>44</t>
+        </is>
+      </c>
+      <c r="E45" s="1" t="inlineStr">
+        <is>
+          <t>entries/c/conservation.md</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>entry_spec_v5</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>source-first v2 inventory; seven checker passes; context-free cold review; blind seal; final reconciliation; 86 targets and 53 relations; 24 source facts</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
         <is>
           <t>true</t>
         </is>
@@ -2523,6 +2783,11 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E38" r:id="rId37"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E39" r:id="rId38"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E40" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E41" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E42" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E43" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E44" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E45" r:id="rId44"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
entry(pose): finalize checked entry after reconciliation
</commit_message>
<xml_diff>
--- a/exports/dictionary_index.xlsx
+++ b/exports/dictionary_index.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J45"/>
+  <dimension ref="A1:J46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -2737,6 +2737,58 @@
         </is>
       </c>
       <c r="J45" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>pose</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>word</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>checked</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>45</t>
+        </is>
+      </c>
+      <c r="E46" s="1" t="inlineStr">
+        <is>
+          <t>entries/p/pose.md</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>entry_spec_v5</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>source-first inventory; seven checker passes; context-free cold review; blind seal; final reconciliation complete</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr">
         <is>
           <t>true</t>
         </is>
@@ -2788,6 +2840,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E43" r:id="rId42"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E44" r:id="rId43"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E45" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E46" r:id="rId45"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
entry(pose): add checked dictionary entry and audit (#121)
Add the checked pose entry, audit artifacts, and synchronized exports.
</commit_message>
<xml_diff>
--- a/exports/dictionary_index.xlsx
+++ b/exports/dictionary_index.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J45"/>
+  <dimension ref="A1:J46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -2737,6 +2737,58 @@
         </is>
       </c>
       <c r="J45" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>pose</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>word</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>checked</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>45</t>
+        </is>
+      </c>
+      <c r="E46" s="1" t="inlineStr">
+        <is>
+          <t>entries/p/pose.md</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>entry_spec_v5</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>source-first inventory; seven checker passes; context-free cold review; blind seal; final reconciliation complete</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr">
         <is>
           <t>true</t>
         </is>
@@ -2788,6 +2840,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E43" r:id="rId42"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E44" r:id="rId43"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E45" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E46" r:id="rId45"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
entry(premise): complete guarded review workflow
</commit_message>
<xml_diff>
--- a/exports/dictionary_index.xlsx
+++ b/exports/dictionary_index.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J46"/>
+  <dimension ref="A1:J47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -2789,6 +2789,58 @@
         </is>
       </c>
       <c r="J46" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>premise</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>word</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>checked</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>46</t>
+        </is>
+      </c>
+      <c r="E47" s="1" t="inlineStr">
+        <is>
+          <t>entries/p/premise.md</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>entry_spec_v5</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>source-first inventory; seven independent checker passes; context-free cold review; secondary zero-finding confirmation; sealed final blind review; final reconciliation passed</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr">
         <is>
           <t>true</t>
         </is>
@@ -2841,6 +2893,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E44" r:id="rId43"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E45" r:id="rId44"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E46" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E47" r:id="rId46"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
entry(premise): add completed dictionary entry
</commit_message>
<xml_diff>
--- a/exports/dictionary_index.xlsx
+++ b/exports/dictionary_index.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J46"/>
+  <dimension ref="A1:J47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -2789,6 +2789,58 @@
         </is>
       </c>
       <c r="J46" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>premise</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>word</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>checked</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>46</t>
+        </is>
+      </c>
+      <c r="E47" s="1" t="inlineStr">
+        <is>
+          <t>entries/p/premise.md</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>entry_spec_v5</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>source-first inventory; seven independent checker passes; context-free cold review; secondary zero-finding confirmation; sealed final blind review; final reconciliation passed</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr">
         <is>
           <t>true</t>
         </is>
@@ -2841,6 +2893,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E44" r:id="rId43"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E45" r:id="rId44"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E46" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E47" r:id="rId46"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
entry(premise): complete final reconciliation
</commit_message>
<xml_diff>
--- a/exports/dictionary_index.xlsx
+++ b/exports/dictionary_index.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J46"/>
+  <dimension ref="A1:J47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -2789,6 +2789,58 @@
         </is>
       </c>
       <c r="J46" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>premise</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>word</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>checked</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>46</t>
+        </is>
+      </c>
+      <c r="E47" s="1" t="inlineStr">
+        <is>
+          <t>entries/p/premise.md</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>entry_spec_v5</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>source-first inventory; seven independent checker passes; context-free cold review; secondary zero-finding confirmation; sealed final blind review; final reconciliation passed</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr">
         <is>
           <t>true</t>
         </is>
@@ -2841,6 +2893,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E44" r:id="rId43"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E45" r:id="rId44"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E46" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E47" r:id="rId46"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
entry(premise): complete audited dictionary entry
Complete the audited premise dictionary entry with source-first and blind-review artifacts.
</commit_message>
<xml_diff>
--- a/exports/dictionary_index.xlsx
+++ b/exports/dictionary_index.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J46"/>
+  <dimension ref="A1:J47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -2789,6 +2789,58 @@
         </is>
       </c>
       <c r="J46" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>premise</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>word</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>checked</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>46</t>
+        </is>
+      </c>
+      <c r="E47" s="1" t="inlineStr">
+        <is>
+          <t>entries/p/premise.md</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>entry_spec_v5</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>source-first inventory; seven independent checker passes; context-free cold review; secondary zero-finding confirmation; sealed final blind review; final reconciliation passed</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr">
         <is>
           <t>true</t>
         </is>
@@ -2841,6 +2893,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E44" r:id="rId43"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E45" r:id="rId44"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E46" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E47" r:id="rId46"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: add desperate dictionary entry and audit
</commit_message>
<xml_diff>
--- a/exports/dictionary_index.xlsx
+++ b/exports/dictionary_index.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J47"/>
+  <dimension ref="A1:J49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -2841,6 +2841,110 @@
         </is>
       </c>
       <c r="J47" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>dimension</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>word</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>checked</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>47</t>
+        </is>
+      </c>
+      <c r="E48" s="1" t="inlineStr">
+        <is>
+          <t>entries/d/dimension.md</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>entry_spec_v5</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>targeted revision: corrected pronunciation; coordinate and rank definitions; sense boundary; torque dimensions; measurements guidance</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>desperate</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>word</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>checked</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>48</t>
+        </is>
+      </c>
+      <c r="E49" s="1" t="inlineStr">
+        <is>
+          <t>entries/d/desperate.md</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>entry_spec_v5</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>mechanical validation; seven checker passes; independent cold review; sealed final blind review; source-first audit; final reconciliation passed</t>
+        </is>
+      </c>
+      <c r="J49" t="inlineStr">
         <is>
           <t>true</t>
         </is>
@@ -2894,6 +2998,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E45" r:id="rId44"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E46" r:id="rId45"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E47" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E48" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E49" r:id="rId48"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: add desperate dictionary entry
Add checked Japanese learner dictionary entry with bounded audit trail.
</commit_message>
<xml_diff>
--- a/exports/dictionary_index.xlsx
+++ b/exports/dictionary_index.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J47"/>
+  <dimension ref="A1:J49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -2841,6 +2841,110 @@
         </is>
       </c>
       <c r="J47" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>dimension</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>word</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>checked</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>47</t>
+        </is>
+      </c>
+      <c r="E48" s="1" t="inlineStr">
+        <is>
+          <t>entries/d/dimension.md</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>entry_spec_v5</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>targeted revision: corrected pronunciation; coordinate and rank definitions; sense boundary; torque dimensions; measurements guidance</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>desperate</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>word</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>checked</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>48</t>
+        </is>
+      </c>
+      <c r="E49" s="1" t="inlineStr">
+        <is>
+          <t>entries/d/desperate.md</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>entry_spec_v5</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>mechanical validation; seven checker passes; independent cold review; sealed final blind review; source-first audit; final reconciliation passed</t>
+        </is>
+      </c>
+      <c r="J49" t="inlineStr">
         <is>
           <t>true</t>
         </is>
@@ -2894,6 +2998,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E45" r:id="rId44"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E46" r:id="rId45"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E47" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E48" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E49" r:id="rId48"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
workflow(scope): seal blind review checkpoint
</commit_message>
<xml_diff>
--- a/exports/dictionary_index.xlsx
+++ b/exports/dictionary_index.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J49"/>
+  <dimension ref="A1:J50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -2945,6 +2945,58 @@
         </is>
       </c>
       <c r="J49" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>scope</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>word</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>checked</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>49</t>
+        </is>
+      </c>
+      <c r="E50" s="1" t="inlineStr">
+        <is>
+          <t>entries/s/scope.md</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>entry_spec_v5</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>source-first inventory; seven independent checker passes; context-free cold review; secondary zero-finding confirmation; sealed final blind review; final reconciliation passed; 216 targets and 156 relations; 27 source facts</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr">
         <is>
           <t>true</t>
         </is>
@@ -3000,6 +3052,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E47" r:id="rId46"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E48" r:id="rId47"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E49" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E50" r:id="rId49"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add checked dictionary entry for scope
Add checked dictionary entry for scope
</commit_message>
<xml_diff>
--- a/exports/dictionary_index.xlsx
+++ b/exports/dictionary_index.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J49"/>
+  <dimension ref="A1:J50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -2945,6 +2945,58 @@
         </is>
       </c>
       <c r="J49" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>scope</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>word</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>checked</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>49</t>
+        </is>
+      </c>
+      <c r="E50" s="1" t="inlineStr">
+        <is>
+          <t>entries/s/scope.md</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>entry_spec_v5</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>source-first inventory; seven independent checker passes; context-free cold review; secondary zero-finding confirmation; sealed final blind review; final reconciliation passed; 216 targets and 156 relations; 27 source facts</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr">
         <is>
           <t>true</t>
         </is>
@@ -3000,6 +3052,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E47" r:id="rId46"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E48" r:id="rId47"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E49" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E50" r:id="rId49"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
workflow(intense): record first audit cycle
</commit_message>
<xml_diff>
--- a/exports/dictionary_index.xlsx
+++ b/exports/dictionary_index.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J50"/>
+  <dimension ref="A1:J52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1199,7 +1199,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>checked</t>
+          <t>needs_review</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -1214,20 +1214,24 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>entry_spec_v1</t>
+          <t>entry_spec_v5</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>true</t>
+          <t>false</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
-        </is>
-      </c>
-      <c r="I16" t="inlineStr"/>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>initial audit rejected; adopted findings require a revised body and one re-audit cycle</t>
+        </is>
+      </c>
       <c r="J16" t="inlineStr">
         <is>
           <t>true</t>
@@ -2997,6 +3001,110 @@
         </is>
       </c>
       <c r="J50" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>publicity</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>word</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>checked</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
+      <c r="E51" s="1" t="inlineStr">
+        <is>
+          <t>entries/p/publicity.md</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>entry_spec_v5</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>source-first inventory; seven independent checker passes; context-free cold review; sealed final blind review; final reconciliation passed; 43 targets; 27 relations; 31 source facts; resolved publicity for/about boundary finding</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>respectively</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>word</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>checked</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>51</t>
+        </is>
+      </c>
+      <c r="E52" s="1" t="inlineStr">
+        <is>
+          <t>entries/r/respectively.md</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>entry_spec_v5</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>source-first inventory; seven independent checker passes; context-free cold review; sealed final blind review; final reconciliation passed; 26 targets and 17 relations; 13 source facts</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr">
         <is>
           <t>true</t>
         </is>
@@ -3053,6 +3161,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E48" r:id="rId47"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E49" r:id="rId48"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E50" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E51" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E52" r:id="rId51"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
entry(intense): complete v5 audit
Repair audit bindings and preserve blind review chronology.
</commit_message>
<xml_diff>
--- a/exports/dictionary_index.xlsx
+++ b/exports/dictionary_index.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J50"/>
+  <dimension ref="A1:J52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1199,7 +1199,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>checked</t>
+          <t>needs_review</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -1214,20 +1214,24 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>entry_spec_v1</t>
+          <t>entry_spec_v5</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>true</t>
+          <t>false</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
-        </is>
-      </c>
-      <c r="I16" t="inlineStr"/>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>sixth-cycle independent final review rejected 7 blockers; revise Oxford level</t>
+        </is>
+      </c>
       <c r="J16" t="inlineStr">
         <is>
           <t>true</t>
@@ -2997,6 +3001,110 @@
         </is>
       </c>
       <c r="J50" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>publicity</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>word</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>checked</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
+      <c r="E51" s="1" t="inlineStr">
+        <is>
+          <t>entries/p/publicity.md</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>entry_spec_v5</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>source-first inventory; seven independent checker passes; context-free cold review; sealed final blind review; final reconciliation passed; 43 targets; 27 relations; 31 source facts; resolved publicity for/about boundary finding</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>respectively</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>word</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>checked</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>51</t>
+        </is>
+      </c>
+      <c r="E52" s="1" t="inlineStr">
+        <is>
+          <t>entries/r/respectively.md</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>entry_spec_v5</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>source-first inventory; seven independent checker passes; context-free cold review; sealed final blind review; final reconciliation passed; 26 targets and 17 relations; 13 source facts</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr">
         <is>
           <t>true</t>
         </is>
@@ -3053,6 +3161,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E48" r:id="rId47"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E49" r:id="rId48"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E50" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E51" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E52" r:id="rId51"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
entry(confine): complete final review
</commit_message>
<xml_diff>
--- a/exports/dictionary_index.xlsx
+++ b/exports/dictionary_index.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J52"/>
+  <dimension ref="A1:J53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1199,7 +1199,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>needs_review</t>
+          <t>checked</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -1219,17 +1219,17 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>false</t>
+          <t>true</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>sixth-cycle independent final review rejected 7 blockers; revise Oxford level</t>
+          <t>zero-based recreation complete; 3 senses</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
@@ -3105,6 +3105,58 @@
         </is>
       </c>
       <c r="J52" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>confine</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>word</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>checked</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>52</t>
+        </is>
+      </c>
+      <c r="E53" s="1" t="inlineStr">
+        <is>
+          <t>entries/c/confine.md</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>entry_spec_v5</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>final review passed; added adjectival confining and source-backed confine A within B coverage</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr">
         <is>
           <t>true</t>
         </is>
@@ -3163,6 +3215,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E50" r:id="rId49"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E51" r:id="rId50"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E52" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E53" r:id="rId52"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
entry(confine): resolve review findings (#146)
Add adjectival confining, source-backed within frames, corrected sense boundaries, completed audit artifacts, and consistent checker request bindings.
</commit_message>
<xml_diff>
--- a/exports/dictionary_index.xlsx
+++ b/exports/dictionary_index.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J52"/>
+  <dimension ref="A1:J53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1199,7 +1199,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>needs_review</t>
+          <t>checked</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -1219,17 +1219,17 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>false</t>
+          <t>true</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>sixth-cycle independent final review rejected 7 blockers; revise Oxford level</t>
+          <t>zero-based recreation complete; 3 senses</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
@@ -3105,6 +3105,58 @@
         </is>
       </c>
       <c r="J52" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>confine</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>word</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>checked</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>52</t>
+        </is>
+      </c>
+      <c r="E53" s="1" t="inlineStr">
+        <is>
+          <t>entries/c/confine.md</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>entry_spec_v5</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>final review passed; added adjectival confining and source-backed confine A within B coverage</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr">
         <is>
           <t>true</t>
         </is>
@@ -3163,6 +3215,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E50" r:id="rId49"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E51" r:id="rId50"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E52" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E53" r:id="rId52"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Finalize reviewed commission dictionary entry
</commit_message>
<xml_diff>
--- a/exports/dictionary_index.xlsx
+++ b/exports/dictionary_index.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J53"/>
+  <dimension ref="A1:J54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -3157,6 +3157,58 @@
         </is>
       </c>
       <c r="J53" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>commission</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>word</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>checked</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>53</t>
+        </is>
+      </c>
+      <c r="E54" s="1" t="inlineStr">
+        <is>
+          <t>entries/c/commission.md</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>entry_spec_v5</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>final review passed; added source-backed delegated-duty sense and unified commercial commission coverage</t>
+        </is>
+      </c>
+      <c r="J54" t="inlineStr">
         <is>
           <t>true</t>
         </is>
@@ -3216,6 +3268,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E51" r:id="rId50"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E52" r:id="rId51"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E53" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E54" r:id="rId53"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Finalize reviewed constitute dictionary entry
</commit_message>
<xml_diff>
--- a/exports/dictionary_index.xlsx
+++ b/exports/dictionary_index.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J54"/>
+  <dimension ref="A1:J55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -3209,6 +3209,58 @@
         </is>
       </c>
       <c r="J54" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>constitute</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>word</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>checked</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>54</t>
+        </is>
+      </c>
+      <c r="E55" s="1" t="inlineStr">
+        <is>
+          <t>entries/c/constitute.md</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>entry_spec_v5</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>source-first inventory; seven independent checker passes and full recheck; context-free cold review; sealed final blind review; final reconciliation passed</t>
+        </is>
+      </c>
+      <c r="J55" t="inlineStr">
         <is>
           <t>true</t>
         </is>
@@ -3269,6 +3321,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E52" r:id="rId51"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E53" r:id="rId52"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E54" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E55" r:id="rId54"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Complete principal workflow and integrate published dictionary entries
</commit_message>
<xml_diff>
--- a/exports/dictionary_index.xlsx
+++ b/exports/dictionary_index.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J54"/>
+  <dimension ref="A1:J56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -3209,6 +3209,110 @@
         </is>
       </c>
       <c r="J54" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>constitute</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>word</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>checked</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>54</t>
+        </is>
+      </c>
+      <c r="E55" s="1" t="inlineStr">
+        <is>
+          <t>entries/c/constitute.md</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>entry_spec_v5</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>source-first inventory; seven independent checker passes and full recheck; context-free cold review; sealed final blind review; final reconciliation passed</t>
+        </is>
+      </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>principal</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>word</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>checked</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>55</t>
+        </is>
+      </c>
+      <c r="E56" s="1" t="inlineStr">
+        <is>
+          <t>entries/p/principal.md</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>entry_spec_v5</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>Independent final review passed; same-run rechecks and final blind completed after removing recheck cap.</t>
+        </is>
+      </c>
+      <c r="J56" t="inlineStr">
         <is>
           <t>true</t>
         </is>
@@ -3269,6 +3373,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E52" r:id="rId51"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E53" r:id="rId52"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E54" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E55" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E56" r:id="rId55"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
entry(principal): finalize checked dictionary entry
</commit_message>
<xml_diff>
--- a/exports/dictionary_index.xlsx
+++ b/exports/dictionary_index.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J54"/>
+  <dimension ref="A1:J55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -3209,6 +3209,58 @@
         </is>
       </c>
       <c r="J54" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>principal</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>word</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>checked</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>55</t>
+        </is>
+      </c>
+      <c r="E55" s="1" t="inlineStr">
+        <is>
+          <t>entries/p/principal.md</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>entry_spec_v5</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>source-first inventory; seven independent checker passes and bounded rechecks; context-free cold review; sealed final blind review; final reconciliation passed</t>
+        </is>
+      </c>
+      <c r="J55" t="inlineStr">
         <is>
           <t>true</t>
         </is>
@@ -3269,6 +3321,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E52" r:id="rId51"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E53" r:id="rId52"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E54" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E55" r:id="rId54"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Finalize magnificent dictionary entry
</commit_message>
<xml_diff>
--- a/exports/dictionary_index.xlsx
+++ b/exports/dictionary_index.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J56"/>
+  <dimension ref="A1:J57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -3313,6 +3313,58 @@
         </is>
       </c>
       <c r="J56" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>magnificent</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>word</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>checked</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>56</t>
+        </is>
+      </c>
+      <c r="E57" s="1" t="inlineStr">
+        <is>
+          <t>entries/m/magnificent.md</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>entry_spec_v5</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>source-first inventory; seven independent checker passes and same-run rechecks; context-free cold review; sealed final blind review; final reconciliation passed</t>
+        </is>
+      </c>
+      <c r="J57" t="inlineStr">
         <is>
           <t>true</t>
         </is>
@@ -3375,6 +3427,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E54" r:id="rId53"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E55" r:id="rId54"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E56" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E57" r:id="rId56"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add checked entry for magnificent (#157)
* workflow(magnificent): initialize guarded run

* Confirm connector workflow checkpoint

* Draft magnificent dictionary entry

* Record magnificent source inventory and review packets

* Record independent magnificent reviews

* Resolve magnificent review findings

* Complete magnificent checker rechecks

* Seal magnificent final blind review

* Record magnificent post-blind context

* Finalize magnificent dictionary entry
</commit_message>
<xml_diff>
--- a/exports/dictionary_index.xlsx
+++ b/exports/dictionary_index.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J56"/>
+  <dimension ref="A1:J57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -3313,6 +3313,58 @@
         </is>
       </c>
       <c r="J56" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>magnificent</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>word</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>checked</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>56</t>
+        </is>
+      </c>
+      <c r="E57" s="1" t="inlineStr">
+        <is>
+          <t>entries/m/magnificent.md</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>entry_spec_v5</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>source-first inventory; seven independent checker passes and same-run rechecks; context-free cold review; sealed final blind review; final reconciliation passed</t>
+        </is>
+      </c>
+      <c r="J57" t="inlineStr">
         <is>
           <t>true</t>
         </is>
@@ -3375,6 +3427,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E54" r:id="rId53"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E55" r:id="rId54"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E56" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E57" r:id="rId56"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add independently reviewed parliament dictionary entry (#158)
* workflow(parliament): initialize guarded run

* Confirm connector workflow checkpoint

* draft(parliament): save generated entry

* audit(parliament): complete source inventory

* review(parliament): resolve findings and recheck entry

* audit(parliament): record final blind handoff

* audit(parliament): seal final blind review

* Complete parliament review revisions and final blind seal

* Fix parliament final resolution body binding

* Finalize parliament source usage binding

* Approve parliament after independent final review
</commit_message>
<xml_diff>
--- a/exports/dictionary_index.xlsx
+++ b/exports/dictionary_index.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J57"/>
+  <dimension ref="A1:J58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -3365,6 +3365,58 @@
         </is>
       </c>
       <c r="J57" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>parliament</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>word</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>checked</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>57</t>
+        </is>
+      </c>
+      <c r="E58" s="1" t="inlineStr">
+        <is>
+          <t>entries/p/parliament.md</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>entry_spec_v5</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>source-first inventory; seven independent checker passes and affected-pass rechecks; context-free cold review; sealed final blind review; final reconciliation passed</t>
+        </is>
+      </c>
+      <c r="J58" t="inlineStr">
         <is>
           <t>true</t>
         </is>
@@ -3428,6 +3480,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E55" r:id="rId54"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E56" r:id="rId55"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E57" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E58" r:id="rId57"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
complete(consequently): mark checked and export
</commit_message>
<xml_diff>
--- a/exports/dictionary_index.xlsx
+++ b/exports/dictionary_index.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J58"/>
+  <dimension ref="A1:J59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -3417,6 +3417,58 @@
         </is>
       </c>
       <c r="J58" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>consequently</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>word</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>checked</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>58</t>
+        </is>
+      </c>
+      <c r="E59" s="1" t="inlineStr">
+        <is>
+          <t>entries/c/consequently.md</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>entry_spec_v5</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>source-first inventory; seven independent checker passes and same-run rechecks; context-free cold review; sealed final blind review; final reconciliation passed</t>
+        </is>
+      </c>
+      <c r="J59" t="inlineStr">
         <is>
           <t>true</t>
         </is>
@@ -3481,6 +3533,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E56" r:id="rId55"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E57" r:id="rId56"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E58" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E59" r:id="rId58"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
workflow(evident): complete final reconciliation
</commit_message>
<xml_diff>
--- a/exports/dictionary_index.xlsx
+++ b/exports/dictionary_index.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J59"/>
+  <dimension ref="A1:J60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -3469,6 +3469,58 @@
         </is>
       </c>
       <c r="J59" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>evident</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>word</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>checked</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>59</t>
+        </is>
+      </c>
+      <c r="E60" s="1" t="inlineStr">
+        <is>
+          <t>entries/e/evident.md</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>entry_spec_v5</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>source-first inventory; seven independent checker passes and affected-pass rechecks; context-free cold review; sealed final blind review; final reconciliation passed</t>
+        </is>
+      </c>
+      <c r="J60" t="inlineStr">
         <is>
           <t>true</t>
         </is>
@@ -3534,6 +3586,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E57" r:id="rId56"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E58" r:id="rId57"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E59" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E60" r:id="rId59"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add evident dictionary entry (#161)
Add the checked evident entry with source-first audit and final review.
</commit_message>
<xml_diff>
--- a/exports/dictionary_index.xlsx
+++ b/exports/dictionary_index.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J59"/>
+  <dimension ref="A1:J60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -3469,6 +3469,58 @@
         </is>
       </c>
       <c r="J59" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>evident</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>word</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>checked</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>59</t>
+        </is>
+      </c>
+      <c r="E60" s="1" t="inlineStr">
+        <is>
+          <t>entries/e/evident.md</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>entry_spec_v5</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>source-first inventory; seven independent checker passes and affected-pass rechecks; context-free cold review; sealed final blind review; final reconciliation passed</t>
+        </is>
+      </c>
+      <c r="J60" t="inlineStr">
         <is>
           <t>true</t>
         </is>
@@ -3534,6 +3586,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E57" r:id="rId56"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E58" r:id="rId57"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E59" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E60" r:id="rId59"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Export sensible dictionary updates
</commit_message>
<xml_diff>
--- a/exports/dictionary_index.xlsx
+++ b/exports/dictionary_index.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J60"/>
+  <dimension ref="A1:J61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -3521,6 +3521,58 @@
         </is>
       </c>
       <c r="J60" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>sensible</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>word</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>checked</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="E61" s="1" t="inlineStr">
+        <is>
+          <t>entries/s/sensible.md</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>entry_spec_v5</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>source-first inventory; seven independent checker passes and affected-pass rechecks; context-free cold review; sealed final blind review; final reconciliation passed</t>
+        </is>
+      </c>
+      <c r="J61" t="inlineStr">
         <is>
           <t>true</t>
         </is>
@@ -3587,6 +3639,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E58" r:id="rId57"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E59" r:id="rId58"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E60" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E61" r:id="rId60"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add sensible dictionary entry (#164)
* workflow(sensible): initialize guarded run

* Confirm connector workflow checkpoint

* Add sensible dictionary entry draft

* Record sensible checker and source audit results

* Record sensible cold review

* Record sensible pre-blind resolution

* Record pre-blind process receipt

* Record sensible checker impact recheck

* Record sensible final blind review

* Seal sensible final blind review

* Record sensible post-blind reconciliation

* Prepare sensible final reconciliation

* Refresh sensible final review inputs

* Mark sensible checked after final review

* Export sensible dictionary updates
</commit_message>
<xml_diff>
--- a/exports/dictionary_index.xlsx
+++ b/exports/dictionary_index.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J60"/>
+  <dimension ref="A1:J61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -3521,6 +3521,58 @@
         </is>
       </c>
       <c r="J60" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>sensible</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>word</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>checked</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="E61" s="1" t="inlineStr">
+        <is>
+          <t>entries/s/sensible.md</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>entry_spec_v5</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>source-first inventory; seven independent checker passes and affected-pass rechecks; context-free cold review; sealed final blind review; final reconciliation passed</t>
+        </is>
+      </c>
+      <c r="J61" t="inlineStr">
         <is>
           <t>true</t>
         </is>
@@ -3587,6 +3639,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E58" r:id="rId57"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E59" r:id="rId58"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E60" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E61" r:id="rId60"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore(audit): stage sealed blind outputs before final review
</commit_message>
<xml_diff>
--- a/exports/dictionary_index.xlsx
+++ b/exports/dictionary_index.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J61"/>
+  <dimension ref="A1:J62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -635,7 +635,6 @@
           <t>2026-06-13</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr"/>
       <c r="J4" t="inlineStr">
         <is>
           <t>true</t>
@@ -735,7 +734,6 @@
           <t>2026-06-13</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr"/>
       <c r="J6" t="inlineStr">
         <is>
           <t>true</t>
@@ -835,7 +833,6 @@
           <t>2026-06-13</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr"/>
       <c r="J8" t="inlineStr">
         <is>
           <t>true</t>
@@ -935,7 +932,6 @@
           <t>2026-06-14</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr"/>
       <c r="J10" t="inlineStr">
         <is>
           <t>true</t>
@@ -983,7 +979,6 @@
           <t>2026-06-14</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr"/>
       <c r="J11" t="inlineStr">
         <is>
           <t>true</t>
@@ -1031,7 +1026,6 @@
           <t>2026-06-14</t>
         </is>
       </c>
-      <c r="I12" t="inlineStr"/>
       <c r="J12" t="inlineStr">
         <is>
           <t>true</t>
@@ -1079,7 +1073,6 @@
           <t>2026-06-14</t>
         </is>
       </c>
-      <c r="I13" t="inlineStr"/>
       <c r="J13" t="inlineStr">
         <is>
           <t>true</t>
@@ -1127,7 +1120,6 @@
           <t>2026-06-14</t>
         </is>
       </c>
-      <c r="I14" t="inlineStr"/>
       <c r="J14" t="inlineStr">
         <is>
           <t>true</t>
@@ -3573,6 +3565,58 @@
         </is>
       </c>
       <c r="J61" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>grant</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>word</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>checked</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="E62" s="1" t="inlineStr">
+        <is>
+          <t>entries/g/grant.md</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>entry_spec_v5</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>source-first inventory; seven independent checker passes; context-free cold review; sealed final blind review; final reconciliation passed</t>
+        </is>
+      </c>
+      <c r="J62" t="inlineStr">
         <is>
           <t>true</t>
         </is>
@@ -3640,6 +3684,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E59" r:id="rId58"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E60" r:id="rId59"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E61" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E62" r:id="rId61"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: add grant dictionary entry (#163)
* chore(audit): stage sealed blind outputs before final review

* fix(audit): restore final review after sealed checkpoint
</commit_message>
<xml_diff>
--- a/exports/dictionary_index.xlsx
+++ b/exports/dictionary_index.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J61"/>
+  <dimension ref="A1:J62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -635,7 +635,6 @@
           <t>2026-06-13</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr"/>
       <c r="J4" t="inlineStr">
         <is>
           <t>true</t>
@@ -735,7 +734,6 @@
           <t>2026-06-13</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr"/>
       <c r="J6" t="inlineStr">
         <is>
           <t>true</t>
@@ -835,7 +833,6 @@
           <t>2026-06-13</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr"/>
       <c r="J8" t="inlineStr">
         <is>
           <t>true</t>
@@ -935,7 +932,6 @@
           <t>2026-06-14</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr"/>
       <c r="J10" t="inlineStr">
         <is>
           <t>true</t>
@@ -983,7 +979,6 @@
           <t>2026-06-14</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr"/>
       <c r="J11" t="inlineStr">
         <is>
           <t>true</t>
@@ -1031,7 +1026,6 @@
           <t>2026-06-14</t>
         </is>
       </c>
-      <c r="I12" t="inlineStr"/>
       <c r="J12" t="inlineStr">
         <is>
           <t>true</t>
@@ -1079,7 +1073,6 @@
           <t>2026-06-14</t>
         </is>
       </c>
-      <c r="I13" t="inlineStr"/>
       <c r="J13" t="inlineStr">
         <is>
           <t>true</t>
@@ -1127,7 +1120,6 @@
           <t>2026-06-14</t>
         </is>
       </c>
-      <c r="I14" t="inlineStr"/>
       <c r="J14" t="inlineStr">
         <is>
           <t>true</t>
@@ -3573,6 +3565,58 @@
         </is>
       </c>
       <c r="J61" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>grant</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>word</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>checked</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="E62" s="1" t="inlineStr">
+        <is>
+          <t>entries/g/grant.md</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>entry_spec_v5</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>source-first inventory; seven independent checker passes; context-free cold review; sealed final blind review; final reconciliation passed</t>
+        </is>
+      </c>
+      <c r="J62" t="inlineStr">
         <is>
           <t>true</t>
         </is>
@@ -3640,6 +3684,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E59" r:id="rId58"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E60" r:id="rId59"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E61" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E62" r:id="rId61"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: add controversial dictionary entry
</commit_message>
<xml_diff>
--- a/exports/dictionary_index.xlsx
+++ b/exports/dictionary_index.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J62"/>
+  <dimension ref="A1:J64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -635,6 +635,7 @@
           <t>2026-06-13</t>
         </is>
       </c>
+      <c r="I4" t="inlineStr"/>
       <c r="J4" t="inlineStr">
         <is>
           <t>true</t>
@@ -734,6 +735,7 @@
           <t>2026-06-13</t>
         </is>
       </c>
+      <c r="I6" t="inlineStr"/>
       <c r="J6" t="inlineStr">
         <is>
           <t>true</t>
@@ -833,6 +835,7 @@
           <t>2026-06-13</t>
         </is>
       </c>
+      <c r="I8" t="inlineStr"/>
       <c r="J8" t="inlineStr">
         <is>
           <t>true</t>
@@ -932,6 +935,7 @@
           <t>2026-06-14</t>
         </is>
       </c>
+      <c r="I10" t="inlineStr"/>
       <c r="J10" t="inlineStr">
         <is>
           <t>true</t>
@@ -979,6 +983,7 @@
           <t>2026-06-14</t>
         </is>
       </c>
+      <c r="I11" t="inlineStr"/>
       <c r="J11" t="inlineStr">
         <is>
           <t>true</t>
@@ -1026,6 +1031,7 @@
           <t>2026-06-14</t>
         </is>
       </c>
+      <c r="I12" t="inlineStr"/>
       <c r="J12" t="inlineStr">
         <is>
           <t>true</t>
@@ -1073,6 +1079,7 @@
           <t>2026-06-14</t>
         </is>
       </c>
+      <c r="I13" t="inlineStr"/>
       <c r="J13" t="inlineStr">
         <is>
           <t>true</t>
@@ -1120,6 +1127,7 @@
           <t>2026-06-14</t>
         </is>
       </c>
+      <c r="I14" t="inlineStr"/>
       <c r="J14" t="inlineStr">
         <is>
           <t>true</t>
@@ -3617,6 +3625,110 @@
         </is>
       </c>
       <c r="J62" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>variation</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>word</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>needs_review</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>61</t>
+        </is>
+      </c>
+      <c r="E63" s="1" t="inlineStr">
+        <is>
+          <t>entries/v/variation.md</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>entry_spec_v5</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>review evidence invalidated; original body and raw records preserved; independent review and known content corrections remain pending</t>
+        </is>
+      </c>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>controversial</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>word</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>checked</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>62</t>
+        </is>
+      </c>
+      <c r="E64" s="1" t="inlineStr">
+        <is>
+          <t>entries/c/controversial.md</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>entry_spec_v5</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>source-first inventory; seven independent checker passes and same-body recheck; context-free cold review; sealed final blind review; final reconciliation passed</t>
+        </is>
+      </c>
+      <c r="J64" t="inlineStr">
         <is>
           <t>true</t>
         </is>
@@ -3685,6 +3797,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E60" r:id="rId59"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E61" r:id="rId60"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E62" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E63" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E64" r:id="rId63"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>